<commit_message>
cambios que estaban pendientes de subir
</commit_message>
<xml_diff>
--- a/calendario_HTML/examples/events.xlsx
+++ b/calendario_HTML/examples/events.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\Curso DAW\02 Segundo\Optativa Python\Proyecto final Juan\calendario_HTML\examples\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD69ECE9-6BC8-4581-A8F4-AA79A6939393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FABEEE5-353C-4E7B-9390-DAB66826E507}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -91,9 +91,6 @@
     <t>De vacaciones en la playa</t>
   </si>
   <si>
-    <t>Tocarme los huevos a dos manos</t>
-  </si>
-  <si>
     <t>relax</t>
   </si>
   <si>
@@ -110,6 +107,9 @@
   </si>
   <si>
     <t>ñaaahh</t>
+  </si>
+  <si>
+    <t>na de na de na</t>
   </si>
 </sst>
 </file>
@@ -539,33 +539,33 @@
         <v>22</v>
       </c>
       <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>24</v>
       </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>25</v>
-      </c>
-      <c r="E6" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
+        <v>26</v>
+      </c>
+      <c r="B7" t="s">
         <v>27</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>28</v>
       </c>
-      <c r="C7" t="s">
-        <v>29</v>
-      </c>
       <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
         <v>25</v>
-      </c>
-      <c r="E7" t="s">
-        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>